<commit_message>
update list of urls
</commit_message>
<xml_diff>
--- a/data/name_and_urls.xlsx
+++ b/data/name_and_urls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lacounty-my.sharepoint.com/personal/mbaker_isd_lacounty_gov/Documents/Desktop/website-status-checker/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{0E81E73B-5DD6-48C7-BBBF-D141271566E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A43430A-93DA-400E-88EF-9715F0EA9BCC}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{156223B0-B841-4D75-8ADC-6B299A3AB2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A33ED2B4-FB30-431C-A16E-940C84C971FD}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E07C0C3F-B82C-4689-BF90-5EF3FEB233FA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
   <si>
     <t>Name</t>
   </si>
@@ -335,9 +335,6 @@
     <t>http://auditor.lacounty.gov</t>
   </si>
   <si>
-    <t>AUDITOR-WIT</t>
-  </si>
-  <si>
     <t>http://wit.lacounty.gov</t>
   </si>
   <si>
@@ -474,6 +471,99 @@
   </si>
   <si>
     <t>http://idco.lacounty.gov</t>
+  </si>
+  <si>
+    <t>https://ballonainterceptor.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://calendar.pw.lacounty.gov/events/</t>
+  </si>
+  <si>
+    <t>https://cleanla.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://equity.pw.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://infrastructurela.org/</t>
+  </si>
+  <si>
+    <t>https://ipm.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://lowerlariver.org</t>
+  </si>
+  <si>
+    <t>https://oilandgas.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://waterforla.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://lacountywomensleadership.org/</t>
+  </si>
+  <si>
+    <t>https://zerowaste.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://ttc.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://mylakids.dcfs.lacounty.gov/</t>
+  </si>
+  <si>
+    <t>https://cbainfo.lacounty.gov</t>
+  </si>
+  <si>
+    <t>https://cannabisdata.lacounty.gov/home/</t>
+  </si>
+  <si>
+    <t>DPW-Zero Waste</t>
+  </si>
+  <si>
+    <t>DPW-Water for LA</t>
+  </si>
+  <si>
+    <t>DPW-Ballona Creek</t>
+  </si>
+  <si>
+    <t>DPW-Infrastructure LA</t>
+  </si>
+  <si>
+    <t>DPW-IPM</t>
+  </si>
+  <si>
+    <t>TTC</t>
+  </si>
+  <si>
+    <t>DPW-Lower LA River</t>
+  </si>
+  <si>
+    <t>DCFS-MyLAKids</t>
+  </si>
+  <si>
+    <t>DPW-Oil and Gas</t>
+  </si>
+  <si>
+    <t>DPW-Equity</t>
+  </si>
+  <si>
+    <t>DPW-Women's Leadership</t>
+  </si>
+  <si>
+    <t>DPW-Clean LA</t>
+  </si>
+  <si>
+    <t>Consumer Business Affairs</t>
+  </si>
+  <si>
+    <t>Cannabis Data</t>
+  </si>
+  <si>
+    <t>DPW-Calendar</t>
+  </si>
+  <si>
+    <t>Auditor-WIT</t>
   </si>
 </sst>
 </file>
@@ -509,8 +599,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -825,10 +918,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5289A946-552F-457A-8BF6-F8D475768729}">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B88"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.6640625" customWidth="1"/>
+    <col min="1" max="1" width="68.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -858,565 +951,688 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>175</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>102</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>173</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>45</v>
+        <v>111</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>113</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>51</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>172</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>158</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>13</v>
+        <v>167</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="B37" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>83</v>
+        <v>162</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>145</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>85</v>
+        <v>174</v>
       </c>
       <c r="B40" t="s">
-        <v>86</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>87</v>
+      <c r="A41" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="B41" t="s">
-        <v>88</v>
+        <v>147</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>117</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>91</v>
+        <v>169</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>149</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>94</v>
+      <c r="A45" s="1" t="s">
+        <v>164</v>
       </c>
       <c r="B45" t="s">
-        <v>95</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>166</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>7</v>
+        <v>168</v>
       </c>
       <c r="B47" t="s">
-        <v>98</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>101</v>
+        <v>161</v>
       </c>
       <c r="B49" t="s">
-        <v>102</v>
+        <v>153</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>103</v>
+        <v>170</v>
       </c>
       <c r="B50" t="s">
-        <v>104</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>105</v>
+        <v>160</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>155</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>11</v>
+        <v>120</v>
       </c>
       <c r="B52" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>112</v>
+        <v>81</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>114</v>
+        <v>14</v>
       </c>
       <c r="B56" t="s">
-        <v>115</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>5</v>
+        <v>126</v>
       </c>
       <c r="B57" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>118</v>
+        <v>61</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="B59" t="s">
-        <v>120</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>121</v>
+        <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>123</v>
+        <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>124</v>
+        <v>63</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="B62" t="s">
-        <v>126</v>
+        <v>86</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>128</v>
+        <v>65</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>3</v>
+        <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>129</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
+        <v>129</v>
+      </c>
+      <c r="B65" t="s">
         <v>130</v>
-      </c>
-      <c r="B65" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>132</v>
+        <v>87</v>
       </c>
       <c r="B66" t="s">
-        <v>133</v>
+        <v>88</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>134</v>
+        <v>89</v>
       </c>
       <c r="B67" t="s">
-        <v>135</v>
+        <v>90</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B68" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="B69" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="B70" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>140</v>
+        <v>9</v>
       </c>
       <c r="B71" t="s">
-        <v>141</v>
+        <v>68</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>142</v>
+        <v>18</v>
       </c>
       <c r="B72" t="s">
-        <v>143</v>
+        <v>69</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
+        <v>80</v>
+      </c>
+      <c r="B73" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>135</v>
+      </c>
+      <c r="B74" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>70</v>
+      </c>
+      <c r="B75" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>2</v>
+      </c>
+      <c r="B76" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>73</v>
+      </c>
+      <c r="B77" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>12</v>
+      </c>
+      <c r="B78" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>94</v>
+      </c>
+      <c r="B79" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>1</v>
+      </c>
+      <c r="B80" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>139</v>
+      </c>
+      <c r="B81" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>13</v>
+      </c>
+      <c r="B82" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>76</v>
+      </c>
+      <c r="B83" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>141</v>
+      </c>
+      <c r="B84" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>96</v>
+      </c>
+      <c r="B85" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>143</v>
+      </c>
+      <c r="B86" t="s">
         <v>144</v>
       </c>
-      <c r="B73" t="s">
-        <v>145</v>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>78</v>
+      </c>
+      <c r="B87" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>165</v>
+      </c>
+      <c r="B88" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B88">
+    <sortCondition ref="A10:A88"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>